<commit_message>
fix product gallery image resolution
</commit_message>
<xml_diff>
--- a/data/catalogo_jusp.xlsx
+++ b/data/catalogo_jusp.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\JUSP\jusp-app2\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19EA6043-9FA2-4F6F-9D58-33943BC3F3E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCB5F206-7097-4A7E-AA7E-A1A312B757DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{9D76B832-63ED-42EE-808B-55D551049E26}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="33">
   <si>
     <t>product_slug</t>
   </si>
@@ -123,6 +123,18 @@
   </si>
   <si>
     <t>Nike Pants Purple</t>
+  </si>
+  <si>
+    <t>nike-dri-fit-quick-dry-running-compression-training-sports-tank-top-women</t>
+  </si>
+  <si>
+    <t>Nike sujetador</t>
+  </si>
+  <si>
+    <t>nike-dunk-low-retro</t>
+  </si>
+  <si>
+    <t>Nike low</t>
   </si>
 </sst>
 </file>
@@ -508,7 +520,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CD597CA-4AEE-4C4B-81F6-85992B5AE07D}">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="12.25" bestFit="1" customWidth="1"/>
@@ -749,6 +761,58 @@
         <v>23</v>
       </c>
     </row>
+    <row r="10" spans="1:8">
+      <c r="A10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E10">
+        <v>99990</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="G10" t="s">
+        <v>23</v>
+      </c>
+      <c r="H10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" t="s">
+        <v>31</v>
+      </c>
+      <c r="B11" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D11">
+        <v>7</v>
+      </c>
+      <c r="E11">
+        <v>99990</v>
+      </c>
+      <c r="F11">
+        <v>1</v>
+      </c>
+      <c r="G11" t="s">
+        <v>24</v>
+      </c>
+      <c r="H11" t="s">
+        <v>24</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
fix product page scope effect loop
</commit_message>
<xml_diff>
--- a/data/catalogo_jusp.xlsx
+++ b/data/catalogo_jusp.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\JUSP\jusp-app2\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D664C317-9EFA-4171-931D-0A9089C77888}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{078D7852-D18D-46F9-9085-BE8482DBAAFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{9D76B832-63ED-42EE-808B-55D551049E26}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="41">
   <si>
     <t>product_slug</t>
   </si>
@@ -672,7 +672,7 @@
         <v>13</v>
       </c>
       <c r="E4">
-        <v>1</v>
+        <v>89990</v>
       </c>
       <c r="F4">
         <v>1</v>
@@ -707,7 +707,7 @@
         <v>14</v>
       </c>
       <c r="E5">
-        <v>1</v>
+        <v>89990</v>
       </c>
       <c r="F5">
         <v>1</v>

</xml_diff>

<commit_message>
fix user orders endpoint
</commit_message>
<xml_diff>
--- a/data/catalogo_jusp.xlsx
+++ b/data/catalogo_jusp.xlsx
@@ -1,42 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\JUSP\jusp-app2\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{078D7852-D18D-46F9-9085-BE8482DBAAFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{9D76B832-63ED-42EE-808B-55D551049E26}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500"/>
   </bookViews>
   <sheets>
     <sheet name="productos" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <si>
     <t>product_slug</t>
   </si>
@@ -56,6 +38,21 @@
     <t>stock</t>
   </si>
   <si>
+    <t>gender</t>
+  </si>
+  <si>
+    <t>category</t>
+  </si>
+  <si>
+    <t>pickup_today</t>
+  </si>
+  <si>
+    <t>express_delivery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">color </t>
+  </si>
+  <si>
     <t>short-nike-kids</t>
   </si>
   <si>
@@ -68,6 +65,15 @@
     <t>XS (135)</t>
   </si>
   <si>
+    <t>kids</t>
+  </si>
+  <si>
+    <t>kisd</t>
+  </si>
+  <si>
+    <t>Black</t>
+  </si>
+  <si>
     <t>S (140)</t>
   </si>
   <si>
@@ -80,6 +86,12 @@
     <t>S</t>
   </si>
   <si>
+    <t>women</t>
+  </si>
+  <si>
+    <t>Pink</t>
+  </si>
+  <si>
     <t>M</t>
   </si>
   <si>
@@ -95,76 +107,46 @@
     <t>S/M</t>
   </si>
   <si>
+    <t>men</t>
+  </si>
+  <si>
+    <t>beige</t>
+  </si>
+  <si>
     <t>M/L</t>
   </si>
   <si>
     <t>L/XL</t>
   </si>
   <si>
-    <t>gender</t>
-  </si>
-  <si>
-    <t>kids</t>
-  </si>
-  <si>
-    <t>women</t>
-  </si>
-  <si>
-    <t>men</t>
-  </si>
-  <si>
-    <t>category</t>
-  </si>
-  <si>
-    <t>kisd</t>
-  </si>
-  <si>
     <t>nike-sports-pants-womens-purple</t>
   </si>
   <si>
+    <t xml:space="preserve">Nike Pants </t>
+  </si>
+  <si>
+    <t>purple</t>
+  </si>
+  <si>
     <t>nike-dri-fit-quick-dry-running-compression-training-sports-tank-top-women</t>
   </si>
   <si>
+    <t>Nike sujetador tops</t>
+  </si>
+  <si>
+    <t>White</t>
+  </si>
+  <si>
     <t>nike-dunk-low-retro</t>
   </si>
   <si>
     <t>Nike low</t>
-  </si>
-  <si>
-    <t>pickup_today</t>
-  </si>
-  <si>
-    <t>express_delivery</t>
-  </si>
-  <si>
-    <t xml:space="preserve">color </t>
-  </si>
-  <si>
-    <t>beige</t>
-  </si>
-  <si>
-    <t>Black</t>
-  </si>
-  <si>
-    <t>Pink</t>
-  </si>
-  <si>
-    <t>White</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nike Pants </t>
-  </si>
-  <si>
-    <t>purple</t>
-  </si>
-  <si>
-    <t>Nike sujetador tops</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <fonts count="2">
     <font>
       <sz val="11"/>
@@ -194,13 +176,7 @@
     </fill>
   </fills>
   <borders count="1">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -216,14 +192,6 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -232,10 +200,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="0E2841"/>
@@ -404,6 +372,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -430,24 +399,25 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="12700" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="19050" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="25400" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -508,52 +478,25 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
-  <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CD597CA-4AEE-4C4B-81F6-85992B5AE07D}">
-  <dimension ref="A1:K11"/>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="30.5" customWidth="1"/>
-    <col min="2" max="2" width="27.08203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.1640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.58203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.08203" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.16406" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.58203" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="14.5">
+    <row r="1" ht="14.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -573,33 +516,33 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="E2">
         <v>88990</v>
@@ -608,10 +551,10 @@
         <v>1</v>
       </c>
       <c r="G2" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="H2" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="I2">
         <v>0</v>
@@ -620,21 +563,21 @@
         <v>0</v>
       </c>
       <c r="K2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C3" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="D3" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="E3">
         <v>88990</v>
@@ -643,10 +586,10 @@
         <v>1</v>
       </c>
       <c r="G3" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="H3" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="I3">
         <v>0</v>
@@ -655,21 +598,21 @@
         <v>0</v>
       </c>
       <c r="K3" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4">
       <c r="A4" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="C4" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="D4" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="E4">
         <v>89990</v>
@@ -678,33 +621,33 @@
         <v>1</v>
       </c>
       <c r="G4" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" t="s">
+        <v>22</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4" t="s">
         <v>23</v>
       </c>
-      <c r="H4" t="s">
-        <v>23</v>
-      </c>
-      <c r="I4">
-        <v>0</v>
-      </c>
-      <c r="J4">
-        <v>0</v>
-      </c>
-      <c r="K4" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11">
+    </row>
+    <row r="5">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="C5" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="D5" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E5">
         <v>89990</v>
@@ -713,45 +656,45 @@
         <v>1</v>
       </c>
       <c r="G5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5" t="s">
         <v>23</v>
       </c>
-      <c r="H5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I5">
-        <v>0</v>
-      </c>
-      <c r="J5">
-        <v>0</v>
-      </c>
-      <c r="K5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11">
+    </row>
+    <row r="6">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="C6" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="D6" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="E6">
         <v>75990</v>
       </c>
       <c r="F6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G6" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="H6" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="I6">
         <v>0</v>
@@ -760,33 +703,33 @@
         <v>0</v>
       </c>
       <c r="K6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="C7" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="D7" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="E7">
         <v>79990</v>
       </c>
       <c r="F7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G7" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="H7" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="I7">
         <v>0</v>
@@ -795,56 +738,56 @@
         <v>0</v>
       </c>
       <c r="K7" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="C8" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="D8" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="E8">
         <v>78990</v>
       </c>
       <c r="F8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G8" t="s">
+        <v>29</v>
+      </c>
+      <c r="H8" t="s">
+        <v>29</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>33</v>
+      </c>
+      <c r="B9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9" t="s">
         <v>24</v>
-      </c>
-      <c r="H8" t="s">
-        <v>24</v>
-      </c>
-      <c r="I8">
-        <v>0</v>
-      </c>
-      <c r="J8">
-        <v>0</v>
-      </c>
-      <c r="K8" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11">
-      <c r="A9" t="s">
-        <v>27</v>
-      </c>
-      <c r="B9" t="s">
-        <v>38</v>
-      </c>
-      <c r="C9" t="s">
-        <v>8</v>
-      </c>
-      <c r="D9" t="s">
-        <v>14</v>
       </c>
       <c r="E9">
         <v>69990</v>
@@ -853,10 +796,10 @@
         <v>1</v>
       </c>
       <c r="G9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I9">
         <v>0</v>
@@ -865,21 +808,21 @@
         <v>0</v>
       </c>
       <c r="K9" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10">
       <c r="A10" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="B10" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C10" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="D10" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E10">
         <v>99990</v>
@@ -888,10 +831,10 @@
         <v>1</v>
       </c>
       <c r="G10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I10">
         <v>0</v>
@@ -900,18 +843,18 @@
         <v>0</v>
       </c>
       <c r="K10" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11">
       <c r="A11" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="B11" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="C11" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="D11">
         <v>7</v>
@@ -923,10 +866,10 @@
         <v>1</v>
       </c>
       <c r="G11" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="H11" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="I11">
         <v>0</v>
@@ -935,10 +878,9 @@
         <v>0</v>
       </c>
       <c r="K11" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: wompi tokenization and direct charge flow
</commit_message>
<xml_diff>
--- a/data/catalogo_jusp.xlsx
+++ b/data/catalogo_jusp.xlsx
@@ -944,10 +944,10 @@
         <v>22</v>
       </c>
       <c r="N2" s="3">
-        <v>46130.833333333328</v>
+        <v>46134</v>
       </c>
       <c r="O2" s="3">
-        <v>46133.957638888889</v>
+        <v>46135</v>
       </c>
       <c r="P2" t="s">
         <v>22</v>

</xml_diff>

<commit_message>
sync: estados dashboard con mis pedidos
</commit_message>
<xml_diff>
--- a/data/catalogo_jusp.xlsx
+++ b/data/catalogo_jusp.xlsx
@@ -1214,7 +1214,7 @@
         <v>21</v>
       </c>
       <c r="L2">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="N2" s="3"/>
       <c r="O2" s="3"/>
@@ -1254,7 +1254,7 @@
         <v>21</v>
       </c>
       <c r="L3">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="N3" s="3"/>
       <c r="O3" s="3"/>

</xml_diff>